<commit_message>
added links and arranged the data in the files
</commit_message>
<xml_diff>
--- a/jpetstore/test_result.xlsx
+++ b/jpetstore/test_result.xlsx
@@ -4,10 +4,10 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" firstSheet="1" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Original Data" sheetId="1" r:id="rId1"/>
+    <sheet name="Original Data" sheetId="1" state="hidden" r:id="rId1"/>
     <sheet name="Test Data" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>

</xml_diff>